<commit_message>
refactor: replace CS with client-owned hybrid networking
Add portable core, room coordinator, LocalUdp/EOS transports, capability state handoff and whole-match resource ownership. Retire the dedicated server target and UE replication paths; keep stable reflected classes and shared gameplay algorithms.

Validation: source UE 5.7 GuLiStrikeEditor Development and core/coordinator Release build successfully. G acceptance remains partial; fault and final performance runs are pending. Temporary captures were excluded from this commit; disk deletion was blocked by tool policy.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeSecondaryWeapons.xlsx
+++ b/data/Excel/GuLiStrikeSecondaryWeapons.xlsx
@@ -1527,7 +1527,7 @@
         <v>189</v>
       </c>
       <c r="L4">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="M4">
         <v>5</v>
@@ -1577,7 +1577,7 @@
         <v>189</v>
       </c>
       <c r="L5">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="M5">
         <v>5</v>
@@ -1750,7 +1750,7 @@
         <v>189</v>
       </c>
       <c r="L9">
-        <v>2400</v>
+        <v>4800</v>
       </c>
       <c r="M9">
         <v>5</v>

</xml_diff>